<commit_message>
incluidas tabelas de resultados
</commit_message>
<xml_diff>
--- a/outputs/jeronimo_google.xlsx
+++ b/outputs/jeronimo_google.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.researchgate.net/profile/Madhusanka-Liyanage/publication/358976899_A_survey_on_Zero_touch_network_and_Service_Management_ZSM_for_5G_and_beyond_networks/links/622065ecadd1b367ae0f6a2a/A-survey-on-Zero-touch-network-and-Service-Management-ZSM-for-5G-and-beyond-networks.pdf</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/6573136/</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://search.ebscohost.com/login.aspx?direct=true&amp;profile=ehost&amp;scope=site&amp;authtype=crawler&amp;jrnl=20856830&amp;AN=157194512&amp;h=AdX86grqA7XRIJXXiqoGYoCCuFy3gaAGefeNT7UVSW%2Bv8pLb1kiW4nY1HBH%2FverqaaxK413vIFVY7UhKJCDADg%3D%3D&amp;crl=c</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.mdpi.com/2079-9292/11/24/4104</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S1389128622001876</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9615540/</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10258188/</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S1389128623005212</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.lntsmartworld.com/assets/img/closed-loop-engine-for-network-automation.pdf</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://eprints.ost.ch/id/eprint/1170/</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/article/10.1007/s10922-020-09517-0</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://repository.uantwerpen.be/link/irua/161998</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9354865/</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10214054/</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://eprints.ost.ch/id/eprint/850/</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.mdpi.com/2079-9292/12/3/566</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9917451/</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.ymatchx.com/c/dam/en/us/products/collateral/cloud-systems-management/network-services-orchestrator/white-paper-sp-ema-trust-in-network-automation.pdf</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://katalog.ub.uni-heidelberg.de/titel/69228141</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9464000/</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10230112/</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9925251/</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10574943/</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/979-8-8688-0391-8_12</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://aaltodoc.aalto.fi/items/1f3d9850-8129-477e-83b0-20ccd5fe1d81</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9983704/</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.researchgate.net/profile/Runwei-Guan/publication/364917224_Traffic_Accident_Scene_Recognition_with_FMCW_Radar_and_Vision_Transformer/links/635e739112cbac6a3e0d0292/Traffic-Accident-Scene-Recognition-with-FMCW-Radar-and-Vision-Transformer.pdf#page=76</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://search.ebscohost.com/login.aspx?direct=true&amp;profile=ehost&amp;scope=site&amp;authtype=crawler&amp;jrnl=20712987&amp;AN=164426624&amp;h=LUK0wHFSGuBB9hxs%2B8B57jsnCx2CjeF9JfZTPoOFEBK0gujPnrkUwlPQ33KVqOQq2Qkl00LRVCEt7%2BNolCaAew%3D%3D&amp;crl=c</t>
         </is>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10461416/</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9482454/</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://books.google.com/books?hl=en&amp;lr=&amp;id=zNfPEAAAQBAJ&amp;oi=fnd&amp;pg=PT40&amp;dq=(%22single+source+of+truth%22+OR+%22source+of+truth%22+OR+%22integrated+network+management%22)+AND+((%22zero+touch+network%22+OR+%22zero-touch+network%22+OR+%22zero+touch+configuration%22+OR+%22zero+touch+management%22+OR+%22zero-touch+management%22)+OR+(%22network+automation%22+OR+%22autonomous+networks%22))&amp;ots=aXEIgQX03m&amp;sig=fe0WVsDqfmr-O-coUfZ_lIsa7_0</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9952437/</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1172,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.scientific.net/AMM.543-547.3036</t>
         </is>
       </c>
     </row>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9789774/</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9919934/</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9464050/</t>
         </is>
       </c>
     </row>
@@ -1278,7 +1278,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://onlinelibrary.wiley.com/doi/abs/10.1002/9781119586449.ch11</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9148441/</t>
         </is>
       </c>
     </row>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/257933/</t>
         </is>
       </c>
     </row>
@@ -1344,7 +1344,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/6573110/</t>
         </is>
       </c>
     </row>
@@ -1366,7 +1366,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9464055/</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dl.acm.org/doi/abs/10.1145/3544216.3544244</t>
         </is>
       </c>
     </row>
@@ -1410,7 +1410,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10012588/</t>
         </is>
       </c>
     </row>
@@ -1432,7 +1432,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S1569190X21001179</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9829768/</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/7140321/</t>
         </is>
       </c>
     </row>
@@ -1498,7 +1498,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://eprints.ost.ch/id/eprint/1151/</t>
         </is>
       </c>
     </row>
@@ -1520,7 +1520,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9464012/</t>
         </is>
       </c>
     </row>
@@ -1542,7 +1542,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9906034/</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10099084/</t>
         </is>
       </c>
     </row>
@@ -1586,7 +1586,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/918034/</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://opg.optica.org/abstract.cfm?uri=OFC-2023-M3Z.8</t>
         </is>
       </c>
     </row>
@@ -1630,7 +1630,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/7140499/</t>
         </is>
       </c>
     </row>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.techrxiv.org/doi/full/10.36227/techrxiv.17075450.v1</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1674,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.igi-global.com/chapter/survey-of-industrial-applications-using-blockchain-and-sixth-generation-network-technology/320331</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0301421508004485</t>
         </is>
       </c>
     </row>
@@ -1718,7 +1718,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.researchgate.net/profile/Adrian-Putley/publication/321199905_Realising_network_intelligence_through_master_data_exploitation_and_dynamic_data_modelling/links/60faf0e81e95fe241a83dc0d/Realising-network-intelligence-through-master-data-exploitation-and-dynamic-data-modelling.pdf</t>
         </is>
       </c>
     </row>
@@ -1740,7 +1740,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://books.google.com/books?hl=en&amp;lr=&amp;id=lsgFEQAAQBAJ&amp;oi=fnd&amp;pg=PT44&amp;dq=(%22single+source+of+truth%22+OR+%22source+of+truth%22+OR+%22integrated+network+management%22)+AND+((%22zero+touch+network%22+OR+%22zero-touch+network%22+OR+%22zero+touch+configuration%22+OR+%22zero+touch+management%22+OR+%22zero-touch+management%22)+OR+(%22network+automation%22+OR+%22autonomous+networks%22))&amp;ots=-nNvmO98Vm&amp;sig=aizcSn5aYFffie4PIbdU4GFP3fc</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.mdpi.com/2079-9292/12/18/3957</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://oak.jejunu.ac.kr/handle/2020.oak/24113</t>
         </is>
       </c>
     </row>
@@ -1806,7 +1806,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://onlinelibrary.wiley.com/doi/abs/10.1002/9781119586449.ch1</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8717791/</t>
         </is>
       </c>
     </row>
@@ -1868,7 +1868,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://onlinelibrary.wiley.com/doi/abs/10.1002/9781119586449.ch7</t>
         </is>
       </c>
     </row>
@@ -1890,7 +1890,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/5188848/</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://conferences.sigcomm.org/sigcomm/2023/files/workshop-snip2/BruyereTuncer_OperatorCentric_SNIP2_nonarchival.pdf</t>
         </is>
       </c>
     </row>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10004899/</t>
         </is>
       </c>
     </row>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dl.acm.org/doi/abs/10.17487/RFC9315</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9464009/</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://doiserbia.nb.rs/Article.aspx?ID=1820-02142400002B</t>
         </is>
       </c>
     </row>
@@ -2022,7 +2022,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9837035/</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://search.proquest.com/openview/2e93abce11ae8d325c84e5a3e9b46d93/1?pq-origsite=gscholar&amp;cbl=32329</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2066,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8893138/</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://icities24.unime.it/papers/33.pdf</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10620685/</t>
         </is>
       </c>
     </row>
@@ -2150,7 +2150,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dl.acm.org/doi/abs/10.1145/3627703.3650086</t>
         </is>
       </c>
     </row>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9921446/</t>
         </is>
       </c>
     </row>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9070195/</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://webthesis.biblio.polito.it/30999/</t>
         </is>
       </c>
     </row>
@@ -2238,7 +2238,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9844074/</t>
         </is>
       </c>
     </row>
@@ -2260,7 +2260,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.academia.edu/download/87878855/Network_Management_Protocols_Analytical_Study_and_Future_Research_Directions.pdf</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10285423/</t>
         </is>
       </c>
     </row>
@@ -2304,7 +2304,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/7934814/</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9464010/</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://koreascience.kr/article/JAKO202419743218091.page</t>
         </is>
       </c>
     </row>
@@ -2370,7 +2370,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://books.google.com/books?hl=en&amp;lr=&amp;id=79i_DwAAQBAJ&amp;oi=fnd&amp;pg=PR4&amp;dq=(%22single+source+of+truth%22+OR+%22source+of+truth%22+OR+%22integrated+network+management%22)+AND+((%22zero+touch+network%22+OR+%22zero-touch+network%22+OR+%22zero+touch+configuration%22+OR+%22zero+touch+management%22+OR+%22zero-touch+management%22)+OR+(%22network+automation%22+OR+%22autonomous+networks%22))&amp;ots=qDgEVKSUdz&amp;sig=KuwooeWPSECPwsi6fATxQ4wZSs4</t>
         </is>
       </c>
     </row>
@@ -2392,7 +2392,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://trepo.tuni.fi/bitstream/handle/10024/153120/NguyenAnh.pdf?sequence=2</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://citeseerx.ist.psu.edu/document?repid=rep1&amp;type=pdf&amp;doi=0956be16b5ae5f26cac05960e52a84871ef1649a</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://elib.its.ac.id/jurnal/jurnalsisfo/submit/index.php/sisfo/article/view/237</t>
         </is>
       </c>
     </row>
@@ -2458,7 +2458,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S2352864820302418</t>
         </is>
       </c>
     </row>
@@ -2480,7 +2480,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/978-981-16-8727-3_2</t>
         </is>
       </c>
     </row>
@@ -2502,7 +2502,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10044186/</t>
         </is>
       </c>
     </row>
@@ -2524,7 +2524,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10040616/</t>
         </is>
       </c>
     </row>
@@ -2546,7 +2546,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9015043/</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://books.google.com/books?hl=en&amp;lr=&amp;id=kzgBEAAAQBAJ&amp;oi=fnd&amp;pg=PA93&amp;dq=(%22single+source+of+truth%22+OR+%22source+of+truth%22+OR+%22integrated+network+management%22)+AND+((%22zero+touch+network%22+OR+%22zero-touch+network%22+OR+%22zero+touch+configuration%22+OR+%22zero+touch+management%22+OR+%22zero-touch+management%22)+OR+(%22network+automation%22+OR+%22autonomous+networks%22))&amp;ots=X9ENS30Lyx&amp;sig=SADS1tSF7J76lREeU6uSx4-4P-U</t>
         </is>
       </c>
     </row>
@@ -2608,7 +2608,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/978-981-19-2868-0_3</t>
         </is>
       </c>
     </row>
@@ -2630,7 +2630,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10154212/</t>
         </is>
       </c>
     </row>
@@ -2652,7 +2652,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10369709/</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10637552/</t>
         </is>
       </c>
     </row>
@@ -2696,7 +2696,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://matheo.uliege.be/handle/2268.2/11524</t>
         </is>
       </c>
     </row>
@@ -2718,7 +2718,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://onlinelibrary.wiley.com/doi/abs/10.1002/9781119586449.ch3</t>
         </is>
       </c>
     </row>
@@ -2740,7 +2740,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://era.library.ualberta.ca/items/37c5f672-53f3-42b0-9e87-f8a783ae4c01/download/6fe2258f-b6dd-42f0-90cd-ced79953f6ef</t>
         </is>
       </c>
     </row>
@@ -2762,7 +2762,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10042484/</t>
         </is>
       </c>
     </row>
@@ -2784,7 +2784,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8620148/</t>
         </is>
       </c>
     </row>
@@ -2806,7 +2806,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://recursos.bps.com.es/files/1205/04.pdf</t>
         </is>
       </c>
     </row>
@@ -2828,7 +2828,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/article/10.1007/s00500-023-09501-1</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://arxiv.org/abs/1907.02278</t>
         </is>
       </c>
     </row>
@@ -2872,7 +2872,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>http://www.intersys-lab.org/media/Deployment%20Considerations%20for%20Information-Centric%20Networking%20(ICN).pdf</t>
         </is>
       </c>
     </row>
@@ -2894,7 +2894,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://womencourage.acm.org/2023/wp-content/uploads/2023/06/womencourage2023-posters-paper72.pdf</t>
         </is>
       </c>
     </row>
@@ -2916,7 +2916,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S1389128621001109</t>
         </is>
       </c>
     </row>
@@ -2938,7 +2938,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://is.muni.cz/th/h920y/System_for_automatic_topology_detection_Archive.pdf</t>
         </is>
       </c>
     </row>
@@ -2960,7 +2960,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8584959/</t>
         </is>
       </c>
     </row>
@@ -2982,7 +2982,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/iel1/49/6541/x0296617.pdf</t>
         </is>
       </c>
     </row>
@@ -3004,7 +3004,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/11568285_9</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.ba-sachsen.de/fileadmin/user_upload/Klymash_Beshlei_development_IT.pdf</t>
         </is>
       </c>
     </row>
@@ -3048,7 +3048,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8787746/</t>
         </is>
       </c>
     </row>
@@ -3070,7 +3070,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.mdpi.com/2076-3417/9/24/5418</t>
         </is>
       </c>
     </row>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://books.google.com/books?hl=en&amp;lr=&amp;id=GN0SEQAAQBAJ&amp;oi=fnd&amp;pg=PA77&amp;dq=(%22single+source+of+truth%22+OR+%22source+of+truth%22+OR+%22integrated+network+management%22)+AND+((%22zero+touch+network%22+OR+%22zero-touch+network%22+OR+%22zero+touch+configuration%22+OR+%22zero+touch+management%22+OR+%22zero-touch+management%22)+OR+(%22network+automation%22+OR+%22autonomous+networks%22))&amp;ots=WoGM6n2x36&amp;sig=olzGucgfHOC5X04SaWDbmia2uFE</t>
         </is>
       </c>
     </row>
@@ -3114,7 +3114,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://arxiv.org/abs/1904.03228</t>
         </is>
       </c>
     </row>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10329588/</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9277893/</t>
         </is>
       </c>
     </row>
@@ -3180,7 +3180,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10056694/</t>
         </is>
       </c>
     </row>
@@ -3202,7 +3202,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10278522/</t>
         </is>
       </c>
     </row>
@@ -3224,7 +3224,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.taylorfrancis.com/chapters/edit/10.1201/9781315220178-13/elements-computational-intelligence-network-management-venkataram</t>
         </is>
       </c>
     </row>
@@ -3246,7 +3246,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9923927/</t>
         </is>
       </c>
     </row>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.academia.edu/download/82190671/pdf.pdf</t>
         </is>
       </c>
     </row>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://search.proquest.com/openview/50e44e354effb60f866130d7d307bc50/1?pq-origsite=gscholar&amp;cbl=18750&amp;diss=y</t>
         </is>
       </c>
     </row>
@@ -3330,7 +3330,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8717852/</t>
         </is>
       </c>
     </row>
@@ -3352,7 +3352,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10384906/</t>
         </is>
       </c>
     </row>
@@ -3374,7 +3374,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.academia.edu/download/62228187/Vol-10-issue-2-M-0120200228-57413-1y0t7y0.pdf</t>
         </is>
       </c>
     </row>
@@ -3396,7 +3396,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://books.google.com/books?hl=en&amp;lr=&amp;id=wtfPEAAAQBAJ&amp;oi=fnd&amp;pg=PT42&amp;dq=(%22single+source+of+truth%22+OR+%22source+of+truth%22+OR+%22integrated+network+management%22)+AND+((%22zero+touch+network%22+OR+%22zero-touch+network%22+OR+%22zero+touch+configuration%22+OR+%22zero+touch+management%22+OR+%22zero-touch+management%22)+OR+(%22network+automation%22+OR+%22autonomous+networks%22))&amp;ots=M2Cd7hoNLx&amp;sig=wBizsy2_7eKXIAngbmLOwk9OeFY</t>
         </is>
       </c>
     </row>
@@ -3418,7 +3418,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9429224/</t>
         </is>
       </c>
     </row>
@@ -3440,7 +3440,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9919594/</t>
         </is>
       </c>
     </row>
@@ -3462,7 +3462,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8717849/</t>
         </is>
       </c>
     </row>
@@ -3484,7 +3484,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>http://users.utcluj.ro/~dobrota/ATN_2_2021_5.pdf</t>
         </is>
       </c>
     </row>
@@ -3506,7 +3506,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://books.google.com/books?hl=en&amp;lr=&amp;id=epvcDgAAQBAJ&amp;oi=fnd&amp;pg=PP1&amp;dq=(%22single+source+of+truth%22+OR+%22source+of+truth%22+OR+%22integrated+network+management%22)+AND+((%22zero+touch+network%22+OR+%22zero-touch+network%22+OR+%22zero+touch+configuration%22+OR+%22zero+touch+management%22+OR+%22zero-touch+management%22)+OR+(%22network+automation%22+OR+%22autonomous+networks%22))&amp;ots=eZ_fSEblpR&amp;sig=mESZ-GXH4KUZ72lOvcodXrkP-4k</t>
         </is>
       </c>
     </row>
@@ -3528,7 +3528,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/978-3-030-26601-1_20</t>
         </is>
       </c>
     </row>
@@ -3550,7 +3550,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/978-3-030-24907-6_10</t>
         </is>
       </c>
     </row>
@@ -3572,7 +3572,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10420937/</t>
         </is>
       </c>
     </row>
@@ -3594,7 +3594,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.scientific.net/AMM.415.34</t>
         </is>
       </c>
     </row>
@@ -3616,7 +3616,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dl.acm.org/doi/abs/10.1145/3512676.3512681</t>
         </is>
       </c>
     </row>
@@ -3638,7 +3638,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://books.google.com/books?hl=en&amp;lr=&amp;id=ttfPEAAAQBAJ&amp;oi=fnd&amp;pg=PP32&amp;dq=(%22single+source+of+truth%22+OR+%22source+of+truth%22+OR+%22integrated+network+management%22)+AND+((%22zero+touch+network%22+OR+%22zero-touch+network%22+OR+%22zero+touch+configuration%22+OR+%22zero+touch+management%22+OR+%22zero-touch+management%22)+OR+(%22network+automation%22+OR+%22autonomous+networks%22))&amp;ots=vm1bzWUQHu&amp;sig=4jcvoDzGhGere-j_jgiJ8Au_kv0</t>
         </is>
       </c>
     </row>
@@ -3660,7 +3660,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8717881/</t>
         </is>
       </c>
     </row>
@@ -3682,7 +3682,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/article/10.1007/s00170-024-14238-8</t>
         </is>
       </c>
     </row>
@@ -3704,7 +3704,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://eprints.ost.ch/id/eprint/1219/1/FS%202024-BA-EP-Bister-Furrer-Green%20Networking%20-%20Visibility,%20a%20first%20step%20towards%20sustaina.pdf</t>
         </is>
       </c>
     </row>
@@ -3726,7 +3726,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ir.lib.uwo.ca/etd/8681/</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3748,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8450000/</t>
         </is>
       </c>
     </row>
@@ -3770,7 +3770,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/978-981-19-2130-8_89</t>
         </is>
       </c>
     </row>
@@ -3792,7 +3792,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://books.google.com/books?hl=en&amp;lr=&amp;id=0tnPEAAAQBAJ&amp;oi=fnd&amp;pg=PT21&amp;dq=(%22single+source+of+truth%22+OR+%22source+of+truth%22+OR+%22integrated+network+management%22)+AND+((%22zero+touch+network%22+OR+%22zero-touch+network%22+OR+%22zero+touch+configuration%22+OR+%22zero+touch+management%22+OR+%22zero-touch+management%22)+OR+(%22network+automation%22+OR+%22autonomous+networks%22))&amp;ots=aRbHWobNcv&amp;sig=Q2Wpp84N8m3lQNDFf2iG1nG98TI</t>
         </is>
       </c>
     </row>
@@ -3814,7 +3814,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/978-3-031-56728-5_45</t>
         </is>
       </c>
     </row>
@@ -3836,7 +3836,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9798822/</t>
         </is>
       </c>
     </row>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://repository.uantwerpen.be/link/irua/192285</t>
         </is>
       </c>
     </row>
@@ -3880,7 +3880,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.taylorfrancis.com/chapters/edit/10.1201/9781032632223-7/blockchain-technology-healthcare-srividhya-pradeepa</t>
         </is>
       </c>
     </row>
@@ -3902,7 +3902,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/7987359/</t>
         </is>
       </c>
     </row>
@@ -3924,7 +3924,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/978-1-4419-6769-5_1</t>
         </is>
       </c>
     </row>
@@ -3946,7 +3946,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8251220/</t>
         </is>
       </c>
     </row>
@@ -3968,7 +3968,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://books.google.com/books?hl=en&amp;lr=&amp;id=HB3qCgAAQBAJ&amp;oi=fnd&amp;pg=PT24&amp;dq=(%22single+source+of+truth%22+OR+%22source+of+truth%22+OR+%22integrated+network+management%22)+AND+((%22zero+touch+network%22+OR+%22zero-touch+network%22+OR+%22zero+touch+configuration%22+OR+%22zero+touch+management%22+OR+%22zero-touch+management%22)+OR+(%22network+automation%22+OR+%22autonomous+networks%22))&amp;ots=Ma58m8Iuf1&amp;sig=vCha_4sp7Wi3WQDz4X70qr_TYy0</t>
         </is>
       </c>
     </row>
@@ -3990,7 +3990,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/content/pdf/10.1007/978-1-4842-7458-3.pdf</t>
         </is>
       </c>
     </row>
@@ -4012,7 +4012,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://theses.hal.science/tel-04612014/</t>
         </is>
       </c>
     </row>
@@ -4034,7 +4034,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.mdpi.com/1424-8220/20/13/3622</t>
         </is>
       </c>
     </row>
@@ -4056,7 +4056,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8464862/</t>
         </is>
       </c>
     </row>
@@ -4078,7 +4078,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dl.acm.org/doi/abs/10.1016/j.comnet.2023.110076</t>
         </is>
       </c>
     </row>
@@ -4100,7 +4100,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://citeseerx.ist.psu.edu/document?repid=rep1&amp;type=pdf&amp;doi=be2581ccb0548cdf6df6e4634d5802da9d1c0d6d</t>
         </is>
       </c>
     </row>
@@ -4122,7 +4122,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10637651/</t>
         </is>
       </c>
     </row>
@@ -4144,7 +4144,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://arxiv.org/abs/2110.12025</t>
         </is>
       </c>
     </row>
@@ -4166,7 +4166,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dl.acm.org/doi/abs/10.1145/3183713.3190653</t>
         </is>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.techrxiv.org/doi/full/10.36227/techrxiv.15176175.v1</t>
         </is>
       </c>
     </row>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10004580/</t>
         </is>
       </c>
     </row>
@@ -4232,7 +4232,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.mdpi.com/2079-9292/13/5/864</t>
         </is>
       </c>
     </row>
@@ -4254,7 +4254,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0140366420305946</t>
         </is>
       </c>
     </row>
@@ -4276,7 +4276,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://webthesis.biblio.polito.it/27748/</t>
         </is>
       </c>
     </row>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://mediatum.ub.tum.de/1463640</t>
         </is>
       </c>
     </row>
@@ -4320,7 +4320,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://resources.geant.org/wp-content/uploads/2023/11/GN5-1_White-Paper_OAV-Maturity-Model.pdf</t>
         </is>
       </c>
     </row>
@@ -4342,7 +4342,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10426261/</t>
         </is>
       </c>
     </row>
@@ -4364,7 +4364,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.publications.scrs.in/uploads/final_menuscript/c7c252d1ff18928a79c9d8ff773dc3a0.pdf</t>
         </is>
       </c>
     </row>
@@ -4386,7 +4386,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.ieice.org/cs/gnl/gnl_vol44-2.pdf#page=13</t>
         </is>
       </c>
     </row>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/7502428/</t>
         </is>
       </c>
     </row>
@@ -4430,7 +4430,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ni4osstor.renam.md:8081/GEANT/GN4-3_White-Paper_OAV-Architectures_v2.0_for_wiki.pdf</t>
         </is>
       </c>
     </row>
@@ -4452,7 +4452,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9625012/</t>
         </is>
       </c>
     </row>
@@ -4474,7 +4474,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://books.google.com/books?hl=en&amp;lr=&amp;id=Uh7_EAAAQBAJ&amp;oi=fnd&amp;pg=PT15&amp;dq=(%22single+source+of+truth%22+OR+%22source+of+truth%22+OR+%22integrated+network+management%22)+AND+((%22zero+touch+network%22+OR+%22zero-touch+network%22+OR+%22zero+touch+configuration%22+OR+%22zero+touch+management%22+OR+%22zero-touch+management%22)+OR+(%22network+automation%22+OR+%22autonomous+networks%22))&amp;ots=eeTK3l4VgB&amp;sig=FYBI69fiYrkyNOSH9On_MbTT6o0</t>
         </is>
       </c>
     </row>
@@ -4496,7 +4496,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://hal.science/hal-04504786/</t>
         </is>
       </c>
     </row>
@@ -4518,7 +4518,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://citeseerx.ist.psu.edu/document?repid=rep1&amp;type=pdf&amp;doi=7baa5dc7bc2e6c95357b06451fa758df04f2a501</t>
         </is>
       </c>
     </row>
@@ -4540,7 +4540,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://jyx.jyu.fi/handle/123456789/75938</t>
         </is>
       </c>
     </row>
@@ -4562,7 +4562,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>http://www.tml.tkk.fi/Research/BBS/IPMAN/internal/doku/</t>
         </is>
       </c>
     </row>
@@ -4584,7 +4584,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ruor.uottawa.ca/handle/10393/44971</t>
         </is>
       </c>
     </row>
@@ -4606,7 +4606,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.researchgate.net/profile/David-Kidston/publication/235120295_Distributed_Network_Management/links/02e7e53c550587ea47000000/Distributed-Network-Management.pdf</t>
         </is>
       </c>
     </row>
@@ -4628,7 +4628,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://par.nsf.gov/biblio/10166357</t>
         </is>
       </c>
     </row>
@@ -4650,7 +4650,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dl.acm.org/doi/abs/10.1145/3176648</t>
         </is>
       </c>
     </row>
@@ -4672,7 +4672,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10107385/</t>
         </is>
       </c>
     </row>
@@ -4694,7 +4694,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://books.google.com/books?hl=en&amp;lr=&amp;id=qppLDwAAQBAJ&amp;oi=fnd&amp;pg=PT35&amp;dq=(%22single+source+of+truth%22+OR+%22source+of+truth%22+OR+%22integrated+network+management%22)+AND+((%22zero+touch+network%22+OR+%22zero-touch+network%22+OR+%22zero+touch+configuration%22+OR+%22zero+touch+management%22+OR+%22zero-touch+management%22)+OR+(%22network+automation%22+OR+%22autonomous+networks%22))&amp;ots=gwtbsevXpP&amp;sig=KsIpwOebJvAvt1p_8WHX_qY8xmQ</t>
         </is>
       </c>
     </row>
@@ -4716,7 +4716,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9059450/</t>
         </is>
       </c>
     </row>
@@ -4738,7 +4738,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://journals.sagepub.com/doi/abs/10.3233/JHS-190601</t>
         </is>
       </c>
     </row>
@@ -4760,7 +4760,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://arxiv.org/abs/2112.14612</t>
         </is>
       </c>
     </row>
@@ -4782,7 +4782,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.comviva.com/wp-content/uploads/2019/12/How_to_leverage_data_WEB.pdf</t>
         </is>
       </c>
     </row>
@@ -4804,7 +4804,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8760495/</t>
         </is>
       </c>
     </row>
@@ -4826,7 +4826,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dl.acm.org/doi/abs/10.1145/2539150.2539267</t>
         </is>
       </c>
     </row>
@@ -4848,7 +4848,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.researchgate.net/profile/Abdurrahman-Hassan-Shuaibu/publication/333703270_Pan_African_International_Confer-_ence_on_Science_Computing_and_Telecommunications_Book_of_Proceedings/links/5cffe64b4585157d15a405f2/Pan-African-International-Confer-ence-on-Science-Computing-and-Telecommunications-Book-of-Proceedings.pdf#page=33</t>
         </is>
       </c>
     </row>
@@ -4870,7 +4870,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.taylorfrancis.com/books/mono/10.1201/9781420064551/advances-network-management-jianguo-ding</t>
         </is>
       </c>
     </row>
@@ -4892,7 +4892,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://books.google.com/books?hl=en&amp;lr=&amp;id=cdkZEQAAQBAJ&amp;oi=fnd&amp;pg=PP1&amp;dq=(%22single+source+of+truth%22+OR+%22source+of+truth%22+OR+%22integrated+network+management%22)+AND+((%22zero+touch+network%22+OR+%22zero-touch+network%22+OR+%22zero+touch+configuration%22+OR+%22zero+touch+management%22+OR+%22zero-touch+management%22)+OR+(%22network+automation%22+OR+%22autonomous+networks%22))&amp;ots=YaGgDtVYJJ&amp;sig=IJMi0ve70_RyEv2IHkWEL7_tXU0</t>
         </is>
       </c>
     </row>
@@ -4914,7 +4914,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://search.proquest.com/openview/f167a8901c320c4e7b30c4eac5eec559/1?pq-origsite=gscholar&amp;cbl=18750&amp;diss=y</t>
         </is>
       </c>
     </row>
@@ -4936,7 +4936,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.mdpi.com/1424-8220/24/3/1038</t>
         </is>
       </c>
     </row>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10347460/</t>
         </is>
       </c>
     </row>
@@ -4980,7 +4980,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/7987334/</t>
         </is>
       </c>
     </row>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9012687/</t>
         </is>
       </c>
     </row>
@@ -5024,7 +5024,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S1084804519302516</t>
         </is>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/7582516/</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.mdpi.com/1424-8220/22/15/5551</t>
         </is>
       </c>
     </row>
@@ -5090,7 +5090,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dl.acm.org/doi/abs/10.1145/3567826</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dspace.lib.uom.gr/handle/2159/30977</t>
         </is>
       </c>
     </row>
@@ -5134,7 +5134,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://jyx.jyu.fi/handle/123456789/52363</t>
         </is>
       </c>
     </row>
@@ -5156,7 +5156,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.emerald.com/insight/content/doi/10.1108/CI-05-2023-0099/full/html</t>
         </is>
       </c>
     </row>
@@ -5178,7 +5178,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8858442/</t>
         </is>
       </c>
     </row>
@@ -5200,7 +5200,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://arxiv.org/abs/2201.03770</t>
         </is>
       </c>
     </row>
@@ -5222,7 +5222,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8388896/</t>
         </is>
       </c>
     </row>
@@ -5244,7 +5244,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0020025514003995</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5266,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ruor.uottawa.ca/items/56a5fea0-5df3-49a8-bc53-d9b8bc8bed09</t>
         </is>
       </c>
     </row>
@@ -5288,7 +5288,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dspace.lib.uom.gr/handle/2159/29632</t>
         </is>
       </c>
     </row>
@@ -5310,7 +5310,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9852048/</t>
         </is>
       </c>
     </row>
@@ -5332,7 +5332,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://repository.library.carleton.ca/concern/etds/nc580n99m</t>
         </is>
       </c>
     </row>
@@ -5354,7 +5354,7 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dl.acm.org/doi/abs/10.1145/3538395.3545314</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5376,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dl.acm.org/doi/abs/10.17487/RFC8568</t>
         </is>
       </c>
     </row>
@@ -5398,7 +5398,7 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://theses.cz/id/p2e5aq/1046_Archive.pdf</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10329947/</t>
         </is>
       </c>
     </row>
@@ -5442,7 +5442,7 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9203354/</t>
         </is>
       </c>
     </row>
@@ -5464,7 +5464,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10386867/</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5486,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S1084804520303489</t>
         </is>
       </c>
     </row>
@@ -5508,7 +5508,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.researchgate.net/profile/Andres-Murillo-2/publication/321008006_SDN_and_NFV_Security_Challenges_for_Integrated_Solutions/links/5c5f1847a6fdccb608b4017b/SDN-and-NFV-Security-Challenges-for-Integrated-Solutions.pdf</t>
         </is>
       </c>
     </row>
@@ -5530,7 +5530,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.researchgate.net/profile/Ranjan-Mazumder/publication/341509854_A_comprehensive_analysis_of_migration_path_towards_open_sourced_SDN_technologies_in_context_of_Network_Orchestration/links/5ec4fc68299bf1c09acc023f/A-comprehensive-analysis-of-migration-path-towards-open-sourced-SDN-technologies-in-context-of-Network-Orchestration.pdf</t>
         </is>
       </c>
     </row>
@@ -5552,7 +5552,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8875715/</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://digitalcommons.jsu.edu/fac_res/171/</t>
         </is>
       </c>
     </row>
@@ -5596,7 +5596,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S1389128620311221</t>
         </is>
       </c>
     </row>
@@ -5618,7 +5618,7 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://library.oapen.org/bitstream/handle/20.500.12657/59385/978-3-031-11089-4.pdf?sequence=1#page=59</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9269043/</t>
         </is>
       </c>
     </row>
@@ -5662,7 +5662,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://estudogeral.uc.pt/retrieve/265460/RicardoFigueiredo_2017254736_vbng.pdf</t>
         </is>
       </c>
     </row>
@@ -5702,7 +5702,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/978-3-319-51966-1_7</t>
         </is>
       </c>
     </row>
@@ -5724,7 +5724,7 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/1020931/</t>
         </is>
       </c>
     </row>
@@ -5746,7 +5746,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/article/10.1007/s12243-024-01036-2</t>
         </is>
       </c>
     </row>
@@ -5768,7 +5768,7 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10060659/</t>
         </is>
       </c>
     </row>
@@ -5790,7 +5790,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://aaltodoc.aalto.fi/items/344b124f-4fd6-4714-83b2-20d426b519b5</t>
         </is>
       </c>
     </row>
@@ -5830,7 +5830,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.researchgate.net/profile/Angelos-Pentelas/publication/375516260_Orchestrating_service_function_chains_over_resource-constrained_network_function_virtualization_NFV_infrastructures/links/654ce7ab3fa26f66f4eab74b/Orchestrating-service-function-chains-over-resource-constrained-network-function-virtualization-NFV-infrastructures.pdf</t>
         </is>
       </c>
     </row>
@@ -5852,7 +5852,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0167739X1730626X</t>
         </is>
       </c>
     </row>
@@ -5874,7 +5874,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8622905/</t>
         </is>
       </c>
     </row>
@@ -5896,7 +5896,7 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.academia.edu/download/97097588/HEPiX_20SDN_NFV_20WG_20Phase_20I_20Report_2010.pdf</t>
         </is>
       </c>
     </row>
@@ -5918,7 +5918,7 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://books.google.com/books?hl=en&amp;lr=&amp;id=yCq_3fzEPrYC&amp;oi=fnd&amp;pg=PR5&amp;dq=(%22single+source+of+truth%22+OR+%22source+of+truth%22+OR+%22integrated+network+management%22)+AND+((%22zero+touch+network%22+OR+%22zero-touch+network%22+OR+%22zero+touch+configuration%22+OR+%22zero+touch+management%22+OR+%22zero-touch+management%22)+OR+(%22network+automation%22+OR+%22autonomous+networks%22))&amp;ots=_KQR3PSiBI&amp;sig=MzClxO9CYC3QpirwI2EEQ9xh_wU</t>
         </is>
       </c>
     </row>
@@ -5940,7 +5940,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dl.acm.org/doi/abs/10.17487/RFC8763</t>
         </is>
       </c>
     </row>
@@ -5962,7 +5962,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.theseus.fi/bitstream/handle/10024/133923/Hoai_Le.pdf?sequence=1</t>
         </is>
       </c>
     </row>
@@ -5984,7 +5984,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8292798/</t>
         </is>
       </c>
     </row>
@@ -6006,7 +6006,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10038472/</t>
         </is>
       </c>
     </row>
@@ -6028,7 +6028,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://openrepository.aut.ac.nz/handle/10292/13544</t>
         </is>
       </c>
     </row>
@@ -6050,7 +6050,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10329927/</t>
         </is>
       </c>
     </row>
@@ -6072,7 +6072,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/article/10.1007/s10922-010-9176-7</t>
         </is>
       </c>
     </row>
@@ -6094,7 +6094,7 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/article/10.1007/s11227-018-2336-3</t>
         </is>
       </c>
     </row>
@@ -6116,7 +6116,7 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S1389128619300131</t>
         </is>
       </c>
     </row>
@@ -6138,7 +6138,7 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8685919/</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6160,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://etda.libraries.psu.edu/catalog/16753hxs376</t>
         </is>
       </c>
     </row>
@@ -6182,7 +6182,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/article/10.1007/s12083-023-01484-y</t>
         </is>
       </c>
     </row>
@@ -6204,7 +6204,7 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://docnum.univ-lorraine.fr/public/DDOC_T_2023_0232_OULAAFFART.pdf</t>
         </is>
       </c>
     </row>
@@ -6226,7 +6226,7 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S1084804516300790</t>
         </is>
       </c>
     </row>
@@ -6248,7 +6248,7 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.theseus.fi/handle/10024/494166</t>
         </is>
       </c>
     </row>
@@ -6270,7 +6270,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://search.ieice.org/bin/summary.php?id=e101-b_2_462</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6292,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://arxiv.org/abs/2312.09355</t>
         </is>
       </c>
     </row>
@@ -6314,7 +6314,7 @@
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10239254/</t>
         </is>
       </c>
     </row>
@@ -6336,7 +6336,7 @@
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/article/10.1007/s11227-023-05392-z</t>
         </is>
       </c>
     </row>
@@ -6358,7 +6358,7 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.scielo.br/j/prod/a/3SZgF7p64sWxPPPXg4RSBkc/</t>
         </is>
       </c>
     </row>
@@ -6380,7 +6380,7 @@
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.mdpi.com/1999-5903/13/3/82</t>
         </is>
       </c>
     </row>
@@ -6402,7 +6402,7 @@
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8806677/</t>
         </is>
       </c>
     </row>
@@ -6424,7 +6424,7 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/article/10.1007/s10796-022-10343-9</t>
         </is>
       </c>
     </row>
@@ -6446,7 +6446,7 @@
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S1389128616304273</t>
         </is>
       </c>
     </row>
@@ -6468,7 +6468,7 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10051839/</t>
         </is>
       </c>
     </row>
@@ -6490,7 +6490,7 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10206040/</t>
         </is>
       </c>
     </row>
@@ -6512,7 +6512,7 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://citeseerx.ist.psu.edu/document?repid=rep1&amp;type=pdf&amp;doi=3fa888113b44ec07bcb636af994878bd628369c3</t>
         </is>
       </c>
     </row>
@@ -6534,7 +6534,7 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10234541/</t>
         </is>
       </c>
     </row>
@@ -6556,7 +6556,7 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/978-3-319-64653-4_3</t>
         </is>
       </c>
     </row>
@@ -6578,7 +6578,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.mdpi.com/2076-3417/12/15/7600</t>
         </is>
       </c>
     </row>
@@ -6600,7 +6600,7 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://repositorio.ufpe.br/handle/123456789/2423</t>
         </is>
       </c>
     </row>
@@ -6622,7 +6622,7 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.locus-project.eu/wp-content/uploads/2021/12/D2.5_nbm_17-11-21.pdf</t>
         </is>
       </c>
     </row>
@@ -6644,7 +6644,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/978-3-319-64653-4_12</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6666,7 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://tsukuba.repo.nii.ac.jp/record/2008222/files/DA010796_abstract.pdf</t>
         </is>
       </c>
     </row>
@@ -6688,7 +6688,7 @@
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0140366421002917</t>
         </is>
       </c>
     </row>
@@ -6710,7 +6710,7 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://search.proquest.com/openview/bd5fe378e5aac0fc1d09d77b66401f24/1?pq-origsite=gscholar&amp;cbl=18750</t>
         </is>
       </c>
     </row>
@@ -6732,7 +6732,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.researchgate.net/profile/Pulkit_Ohri/publication/369842495_Software-Defined_Networking_Security_Challenges_and_Solutions_A_Comprehensive_Survey/links/6499584cc41fb852dd340ed7/Software-Defined-Networking-Security-Challenges-and-Solutions-A-Comprehensive-Survey.pdf</t>
         </is>
       </c>
     </row>
@@ -6754,7 +6754,7 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.researchsquare.com/article/rs-3347362/latest</t>
         </is>
       </c>
     </row>
@@ -6776,7 +6776,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8931372/</t>
         </is>
       </c>
     </row>
@@ -6798,7 +6798,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8442690/</t>
         </is>
       </c>
     </row>
@@ -6820,7 +6820,7 @@
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://onlinelibrary.wiley.com/doi/abs/10.1002/9781394216147.ch6</t>
         </is>
       </c>
     </row>
@@ -6842,7 +6842,7 @@
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/B9780128165027000178</t>
         </is>
       </c>
     </row>
@@ -6864,7 +6864,7 @@
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://epub.fh-joanneum.at/obvfhjhs/content/titleinfo/9300521/full.pdf</t>
         </is>
       </c>
     </row>
@@ -6886,7 +6886,7 @@
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://search.proquest.com/openview/e315cda4e5bbc9a2a38d7a684e14b671/1?pq-origsite=gscholar&amp;cbl=2026366&amp;diss=y</t>
         </is>
       </c>
     </row>
@@ -6908,7 +6908,7 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/article/10.1007/s10922-023-09732-5</t>
         </is>
       </c>
     </row>
@@ -6930,7 +6930,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9165408/</t>
         </is>
       </c>
     </row>
@@ -6952,7 +6952,7 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://upcommons.upc.edu/handle/2117/105813</t>
         </is>
       </c>
     </row>
@@ -6974,7 +6974,7 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S1084804516303186</t>
         </is>
       </c>
     </row>
@@ -6996,7 +6996,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S1084804521001569</t>
         </is>
       </c>
     </row>
@@ -7018,7 +7018,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.academia.edu/download/77686590/Thesis.pdf</t>
         </is>
       </c>
     </row>
@@ -7040,7 +7040,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10391345/</t>
         </is>
       </c>
     </row>
@@ -7062,7 +7062,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.scientific.net/AMM.631-632.864</t>
         </is>
       </c>
     </row>
@@ -7084,7 +7084,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10423393/</t>
         </is>
       </c>
     </row>
@@ -7106,7 +7106,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://core.ac.uk/download/pdf/197482188.pdf</t>
         </is>
       </c>
     </row>
@@ -7128,7 +7128,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>http://www.tml.hut.fi/Tutkimus/G4/data/ipman/documents/metsodiploma.pdf</t>
         </is>
       </c>
     </row>
@@ -7150,7 +7150,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://vb.mruni.eu/object/elaba:151958947/</t>
         </is>
       </c>
     </row>
@@ -7172,7 +7172,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.tdx.cat/handle/10803/403990</t>
         </is>
       </c>
     </row>
@@ -7194,7 +7194,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dl.acm.org/doi/abs/10.1145/1506270.1506399</t>
         </is>
       </c>
     </row>
@@ -7216,7 +7216,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.taylorfrancis.com/chapters/edit/10.1201/9781003145721-4/flow-table-scalability-software-defined-networking-brief-overview-abinas-panda-ashok-kumar-turuk-aliva-panda-tarinee-prasad-sahoo-ankit-aryan-kshira-sagar-sahoo</t>
         </is>
       </c>
     </row>
@@ -7238,7 +7238,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9209606/</t>
         </is>
       </c>
     </row>
@@ -7260,7 +7260,7 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S108480451730317X</t>
         </is>
       </c>
     </row>
@@ -7282,7 +7282,7 @@
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/978-3-031-26507-5_15</t>
         </is>
       </c>
     </row>
@@ -7304,7 +7304,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://upcommons.upc.edu/handle/2117/129242</t>
         </is>
       </c>
     </row>
@@ -7326,7 +7326,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/11880905_6</t>
         </is>
       </c>
     </row>
@@ -7348,7 +7348,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.mdpi.com/1999-5903/10/3/23</t>
         </is>
       </c>
     </row>
@@ -7370,7 +7370,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://citeseerx.ist.psu.edu/document?repid=rep1&amp;type=pdf&amp;doi=0f9da7d0e2c2011d1a4c2e63bdfc33ebb92669a3</t>
         </is>
       </c>
     </row>
@@ -7392,7 +7392,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S1389128616302407</t>
         </is>
       </c>
     </row>
@@ -7414,7 +7414,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>http://wipkip.nikhef.nl/events/defcon/DEF%20CON%2022/DEF%20CON%2022%20presentations/Dhia%20Mahjoub,%20Andree%20Toonk,%20and%20Thibault%20Reuille%20-%20Updated/DEFCON-22-Mahjoub-Reuille-Toonk-Catching-Malware-En-Masse-DNS-IP-Style-WP.pdf</t>
         </is>
       </c>
     </row>
@@ -7436,7 +7436,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.mdpi.com/1424-8220/20/3/828</t>
         </is>
       </c>
     </row>
@@ -7458,7 +7458,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.taylorfrancis.com/chapters/edit/10.1201/9780429424878-17/secure-fault-tolerant-computing-mobile-ad-hoc-networks-parmeet-kaur-awadhesh-kumar-singh</t>
         </is>
       </c>
     </row>
@@ -7480,7 +7480,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10621159/</t>
         </is>
       </c>
     </row>
@@ -7502,7 +7502,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://books.google.com/books?hl=en&amp;lr=&amp;id=8Sc-DwAAQBAJ&amp;oi=fnd&amp;pg=PA75&amp;dq=(%22single+source+of+truth%22+OR+%22source+of+truth%22+OR+%22integrated+network+management%22)+AND+((%22zero+touch+network%22+OR+%22zero-touch+network%22+OR+%22zero+touch+configuration%22+OR+%22zero+touch+management%22+OR+%22zero-touch+management%22)+OR+(%22network+automation%22+OR+%22autonomous+networks%22))&amp;ots=6oZpTQmzpp&amp;sig=BvicIPEZC_ZYtSFDDLymXY5Jc-s</t>
         </is>
       </c>
     </row>
@@ -7524,7 +7524,7 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S1389128624002871</t>
         </is>
       </c>
     </row>
@@ -7546,7 +7546,7 @@
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://api.taylorfrancis.com/content/books/mono/download?identifierName=doi&amp;identifierValue=10.1201/9781315220178&amp;type=googlepdf</t>
         </is>
       </c>
     </row>
@@ -7568,7 +7568,7 @@
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9238872/</t>
         </is>
       </c>
     </row>
@@ -7608,7 +7608,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/978-3-319-18467-8_42</t>
         </is>
       </c>
     </row>
@@ -7630,7 +7630,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.researchgate.net/profile/Carolina-Fortuna/publication/359722523_AI-Enabled_Life_Cycle_Automation_of_Smart_Infrastructures/links/624b5c0b5e2f8c7a035a4fe7/AI-Enabled-Life-Cycle-Automation-of-Smart-Infrastructures.pdf</t>
         </is>
       </c>
     </row>
@@ -7652,7 +7652,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.emerald.com/insight/content/doi/10.1108/SASBE-12-2023-0389/full/html</t>
         </is>
       </c>
     </row>
@@ -7674,7 +7674,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10136039/</t>
         </is>
       </c>
     </row>
@@ -7696,7 +7696,7 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://search.proquest.com/openview/7c31479c59c68011da65ffe59c06eac7/1?pq-origsite=gscholar&amp;cbl=18750&amp;diss=y</t>
         </is>
       </c>
     </row>
@@ -7718,7 +7718,7 @@
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ntnuopen.ntnu.no/ntnu-xmlui/handle/11250/2489341</t>
         </is>
       </c>
     </row>
@@ -7740,7 +7740,7 @@
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://open.uct.ac.za/handle/11427/30923</t>
         </is>
       </c>
     </row>
@@ -7762,7 +7762,7 @@
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://scholarworks.calstate.edu/downloads/05742040x</t>
         </is>
       </c>
     </row>
@@ -7784,7 +7784,7 @@
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8384185/</t>
         </is>
       </c>
     </row>
@@ -7806,7 +7806,7 @@
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ntnuopen.ntnu.no/ntnu-xmlui/handle/11250/3133782</t>
         </is>
       </c>
     </row>
@@ -7828,7 +7828,7 @@
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://espace.etsmtl.ca/id/eprint/1938/</t>
         </is>
       </c>
     </row>
@@ -7850,7 +7850,7 @@
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.mdpi.com/1424-8220/23/7/3395</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.researchgate.net/profile/Ali-Malik-4/publication/356387843_A_Survey_of_Machine_Learning_Techniques_for_Video_Quality_Prediction_from_Quality_of_Delivery_Metrics/links/6197aa45d7d1af224b07bae2/A-Survey-of-Machine-Learning-Techniques-for-Video-Quality-Prediction-from-Quality-of-Delivery-Metrics.pdf</t>
         </is>
       </c>
     </row>
@@ -7894,7 +7894,7 @@
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.mdpi.com/2078-2489/14/4/209</t>
         </is>
       </c>
     </row>
@@ -7916,7 +7916,7 @@
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://open.uct.ac.za/handle/11427/5153</t>
         </is>
       </c>
     </row>
@@ -7938,7 +7938,7 @@
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.academia.edu/download/67449245/43_22852_EM_26oct_20oct_11apr_N_Single_Author_.pdf</t>
         </is>
       </c>
     </row>
@@ -7960,7 +7960,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.taylorfrancis.com/chapters/edit/10.1201/9780429424878-21/role-software-defined-networking-sdn-internet-things-iot-security-attacks-countermeasures-megha-quamara-brij-gupta</t>
         </is>
       </c>
     </row>
@@ -7982,7 +7982,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9685093/</t>
         </is>
       </c>
     </row>
@@ -8004,7 +8004,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://arrow.tudublin.ie/engdoc/141/</t>
         </is>
       </c>
     </row>
@@ -8026,7 +8026,7 @@
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://search.proquest.com/openview/3600a579a8d4fa5964fc2c6df4d4f6a0/1?pq-origsite=gscholar&amp;cbl=18750&amp;diss=y</t>
         </is>
       </c>
     </row>
@@ -8048,7 +8048,7 @@
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://itcon.org/papers/2024_21-ITcon-Toyin.pdf</t>
         </is>
       </c>
     </row>
@@ -8070,7 +8070,7 @@
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://books.google.com/books?hl=en&amp;lr=&amp;id=_3ezEAAAQBAJ&amp;oi=fnd&amp;pg=PP1&amp;dq=(%22single+source+of+truth%22+OR+%22source+of+truth%22+OR+%22integrated+network+management%22)+AND+((%22zero+touch+network%22+OR+%22zero-touch+network%22+OR+%22zero+touch+configuration%22+OR+%22zero+touch+management%22+OR+%22zero-touch+management%22)+OR+(%22network+automation%22+OR+%22autonomous+networks%22))&amp;ots=Zeqe3IAn6L&amp;sig=cauHGWuSRyglsgqSfybbpHzoNkc</t>
         </is>
       </c>
     </row>
@@ -8092,7 +8092,7 @@
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://onlinelibrary.wiley.com/doi/abs/10.1002/9781119675525.ch2</t>
         </is>
       </c>
     </row>
@@ -8114,7 +8114,7 @@
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/978-3-031-37920-8_2</t>
         </is>
       </c>
     </row>
@@ -8136,7 +8136,7 @@
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.tandfonline.com/doi/abs/10.1080/01446193.2022.2056216</t>
         </is>
       </c>
     </row>
@@ -8176,7 +8176,7 @@
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.mdpi.com/2079-9292/10/22/2851</t>
         </is>
       </c>
     </row>
@@ -8198,7 +8198,7 @@
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9665016/</t>
         </is>
       </c>
     </row>
@@ -8220,7 +8220,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://scholarworks.montana.edu/items/88e87865-8518-4165-8e55-3e4969c3a0f4</t>
         </is>
       </c>
     </row>
@@ -8242,7 +8242,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.atlantis-press.com/proceedings/amee-17/25883931</t>
         </is>
       </c>
     </row>
@@ -8264,7 +8264,7 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0167739X18302322</t>
         </is>
       </c>
     </row>
@@ -8286,7 +8286,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/10571101/</t>
         </is>
       </c>
     </row>
@@ -8308,7 +8308,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/6171992/</t>
         </is>
       </c>
     </row>
@@ -8330,7 +8330,7 @@
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://search.proquest.com/openview/82eb420d6dc68d0be01b04e88f429bd0/1?pq-origsite=gscholar&amp;cbl=18750&amp;diss=y</t>
         </is>
       </c>
     </row>
@@ -8352,7 +8352,7 @@
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dl.acm.org/doi/abs/10.1016/j.comnet.2023.110016</t>
         </is>
       </c>
     </row>
@@ -8374,7 +8374,7 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.techrxiv.org/doi/full/10.36227/techrxiv.18857759.v1</t>
         </is>
       </c>
     </row>
@@ -8414,7 +8414,7 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.mdpi.com/2079-9292/11/14/2245</t>
         </is>
       </c>
     </row>
@@ -8436,7 +8436,7 @@
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/7810967/</t>
         </is>
       </c>
     </row>
@@ -8458,7 +8458,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://stage.resources.geant.org/wp-content/uploads/2022/02/D6-2_Automation-and-Orchestration-of-Services-in-the-GEANT-Community.pdf</t>
         </is>
       </c>
     </row>
@@ -8480,7 +8480,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://search.proquest.com/openview/4255c948b5164120ee7363052ebff5cb/1?pq-origsite=gscholar&amp;cbl=18750&amp;diss=y</t>
         </is>
       </c>
     </row>
@@ -8502,7 +8502,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://journal.info.unlp.edu.ar/JCST/article/view/736</t>
         </is>
       </c>
     </row>
@@ -8524,7 +8524,7 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/BFb0013901</t>
         </is>
       </c>
     </row>
@@ -8546,7 +8546,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=4259999</t>
         </is>
       </c>
     </row>
@@ -8568,7 +8568,7 @@
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://espace.curtin.edu.au/handle/20.500.11937/89463</t>
         </is>
       </c>
     </row>
@@ -8590,7 +8590,7 @@
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/978-3-030-49190-1_8</t>
         </is>
       </c>
     </row>
@@ -8612,7 +8612,7 @@
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.inderscienceonline.com/doi/abs/10.1504/IJBC.2023.138377</t>
         </is>
       </c>
     </row>
@@ -8634,7 +8634,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.academia.edu/download/110901067/4067186.pdf</t>
         </is>
       </c>
     </row>
@@ -8656,7 +8656,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8406172/</t>
         </is>
       </c>
     </row>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://search.proquest.com/openview/7e9801e3edfba1d50768488bd2984fab/1?pq-origsite=gscholar&amp;cbl=18750</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="D379" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://books.google.com/books?hl=en&amp;lr=&amp;id=i3xZEAAAQBAJ&amp;oi=fnd&amp;pg=PP1&amp;dq=(%22single+source+of+truth%22+OR+%22source+of+truth%22+OR+%22integrated+network+management%22)+AND+((%22zero+touch+network%22+OR+%22zero-touch+network%22+OR+%22zero+touch+configuration%22+OR+%22zero+touch+management%22+OR+%22zero-touch+management%22)+OR+(%22network+automation%22+OR+%22autonomous+networks%22))&amp;ots=KJv1GhNmqz&amp;sig=NSWA1uaAO5V9SLA4Cqlj_85COPU</t>
         </is>
       </c>
     </row>
@@ -8740,7 +8740,7 @@
       </c>
       <c r="D380" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.sciencedirect.com/science/article/pii/S0950584908001389</t>
         </is>
       </c>
     </row>
@@ -8762,7 +8762,7 @@
       </c>
       <c r="D381" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.diva-portal.org/smash/get/diva2:1078159/FULLTEXT02</t>
         </is>
       </c>
     </row>
@@ -8784,7 +8784,7 @@
       </c>
       <c r="D382" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://search.proquest.com/openview/9e86842fa4c711680d675baf74546969/1?pq-origsite=gscholar&amp;cbl=18750&amp;diss=y</t>
         </is>
       </c>
     </row>
@@ -8806,7 +8806,7 @@
       </c>
       <c r="D383" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.theseus.fi/handle/10024/794230</t>
         </is>
       </c>
     </row>
@@ -8828,7 +8828,7 @@
       </c>
       <c r="D384" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://link.springer.com/chapter/10.1007/978-981-19-7395-6_3</t>
         </is>
       </c>
     </row>
@@ -8850,7 +8850,7 @@
       </c>
       <c r="D385" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/9978863/</t>
         </is>
       </c>
     </row>
@@ -8872,7 +8872,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://search.proquest.com/openview/1e4a9069c801e356c11eb7f2a4e7eeee/1?pq-origsite=gscholar&amp;cbl=2026366&amp;diss=y</t>
         </is>
       </c>
     </row>
@@ -8894,7 +8894,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://onlinelibrary.wiley.com/doi/abs/10.1002/0470846119.ch4</t>
         </is>
       </c>
     </row>
@@ -8916,7 +8916,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dspace.cuni.cz/handle/20.500.11956/177594</t>
         </is>
       </c>
     </row>
@@ -8938,7 +8938,7 @@
       </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.cs.kuleuven.be/publicaties/rapporten/cw/CW485.pdf</t>
         </is>
       </c>
     </row>
@@ -8960,7 +8960,7 @@
       </c>
       <c r="D390" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.theseus.fi/bitstream/handle/10024/506961/Vainola_Lassi.pdf?sequence=2</t>
         </is>
       </c>
     </row>
@@ -8982,7 +8982,7 @@
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://library.oapen.org/handle/20.500.12657/42480</t>
         </is>
       </c>
     </row>
@@ -9004,7 +9004,7 @@
       </c>
       <c r="D392" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>http://chipts.ucla.edu/wp-content/uploads/2011/10/Estrin-CV.pdf</t>
         </is>
       </c>
     </row>
@@ -9026,7 +9026,7 @@
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ieeexplore.ieee.org/abstract/document/8406117/</t>
         </is>
       </c>
     </row>
@@ -9048,7 +9048,7 @@
       </c>
       <c r="D394" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.rfc-editor.org/rfc/rfc8568.html</t>
         </is>
       </c>
     </row>
@@ -9070,7 +9070,7 @@
       </c>
       <c r="D395" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://scholar.archive.org/work/hezvdqf2ujbank3wa2gmje3w4m/access/wayback/http://dpi-proceedings.com/index.php/dtcse/article/download/5745/5363</t>
         </is>
       </c>
     </row>
@@ -9092,7 +9092,7 @@
       </c>
       <c r="D396" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.usenix.org/system/files/login/issues/login12-02.pdf</t>
         </is>
       </c>
     </row>
@@ -9114,7 +9114,7 @@
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://eprints.ost.ch/id/eprint/975/</t>
         </is>
       </c>
     </row>
@@ -9136,7 +9136,7 @@
       </c>
       <c r="D398" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://eprints.ost.ch/id/eprint/986/1/HS%202021%202022-BA-EP-Steudler-Kubli-Kraken%202.0.pdf</t>
         </is>
       </c>
     </row>
@@ -9158,7 +9158,7 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://cyberleninka.ru/article/n/bezopasnyy-obmen-faylami-na-osnove-setey-doveriya-i-sertifikatov-otkrytyh-klyuchey-s-pomoschyu-razrabotannogo-prilozheniya</t>
         </is>
       </c>
     </row>
@@ -9180,7 +9180,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://eprints.ost.ch/id/eprint/734/1/HS%202018%202019-SA-EP-Zwicker-Wenk-LAB%20Builder%20mit%20ACI.pdf</t>
         </is>
       </c>
     </row>
@@ -9202,7 +9202,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://ekmair.ukma.edu.ua/bitstream/123456789/22031/1/Nakytniak_Bakalavrska_robota.pdf</t>
         </is>
       </c>
     </row>
@@ -9224,7 +9224,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://rielac.cujae.edu.cu/index.php/rieac/article/view/952</t>
         </is>
       </c>
     </row>
@@ -9246,7 +9246,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://eprints.ost.ch/id/eprint/1013/1/HS%202021%202022-SA-EP-Martinez-Grimm-Software-Entwicklung%20in%20der%20Netzwerk-Automatisierung%20(1).pdf</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="D404" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://webthesis.biblio.polito.it/22651/</t>
         </is>
       </c>
     </row>
@@ -9290,7 +9290,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://otik.uk.zcu.cz/handle/11025/57242</t>
         </is>
       </c>
     </row>
@@ -9312,7 +9312,7 @@
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.jstage.jst.go.jp/article/nictkenkyuhoukoku/64/2/64_85/_article/-char/ja/</t>
         </is>
       </c>
     </row>
@@ -9334,7 +9334,7 @@
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://www.jstage.jst.go.jp/article/bplus/12/1/12_29/_article/-char/ja/</t>
         </is>
       </c>
     </row>
@@ -9356,7 +9356,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://eprints.ost.ch/id/eprint/690/</t>
         </is>
       </c>
     </row>
@@ -9378,7 +9378,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dspace.unipampa.edu.br/handle/riu/8650</t>
         </is>
       </c>
     </row>
@@ -9400,7 +9400,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>http://digital-economy.ru/images/easyblog_articles/1121/tnet456546.pdf</t>
         </is>
       </c>
     </row>
@@ -9422,7 +9422,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://webthesis.biblio.polito.it/secure/16731/1/tesi.pdf</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9444,7 @@
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://dspace.cvut.cz/handle/10467/109776</t>
         </is>
       </c>
     </row>
@@ -9466,7 +9466,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://epub.fh-joanneum.at/obvfhjhs/content/titleinfo/8625465/full.pdf</t>
         </is>
       </c>
     </row>
@@ -9488,7 +9488,7 @@
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://search.proquest.com/openview/85b1920d079f5cfcc44fdf1b15e855aa/1?pq-origsite=gscholar&amp;cbl=2026366&amp;diss=y</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://xuebao.neu.edu.cn/natural/CN/10.12068/j.issn.1005-3026.2002.01.007</t>
         </is>
       </c>
     </row>
@@ -9532,7 +9532,7 @@
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>http://scielo.sld.cu/scielo.php?pid=S1815-59282022000300001&amp;script=sci_arttext&amp;tlng=en</t>
         </is>
       </c>
     </row>
@@ -9554,7 +9554,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://rua.ua.es/dspace/handle/10045/116684</t>
         </is>
       </c>
     </row>
@@ -9576,7 +9576,7 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>http://dspace1.univ-tlemcen.dz/bitstream/112/19056/1/Ms.Tel.Madouri%2BKechkeche.pdf</t>
         </is>
       </c>
     </row>
@@ -9598,7 +9598,7 @@
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://core.ac.uk/download/pdf/85128157.pdf</t>
         </is>
       </c>
     </row>
@@ -9620,7 +9620,7 @@
       </c>
       <c r="D420" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://theses.hal.science/tel-02110343/</t>
         </is>
       </c>
     </row>
@@ -9642,7 +9642,7 @@
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t>NoURL</t>
+          <t>https://repositorio.ipv.pt/handle/10400.19/8348</t>
         </is>
       </c>
     </row>

</xml_diff>